<commit_message>
Implement Sprint 2 store accounts and verification
</commit_message>
<xml_diff>
--- a/acceptance_matrix.xlsx
+++ b/acceptance_matrix.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="1" r:id="R7c30f09fb1684ccc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Summary" sheetId="2" r:id="R1d1959c6f94149f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Personas" sheetId="3" r:id="R3cafc28c00774d7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Traceability" sheetId="4" r:id="Rceb6a90ece6340d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="1" r:id="R26a23ca8bdf84be9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Summary" sheetId="2" r:id="R5eb59a6c0bd94122"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Personas" sheetId="3" r:id="R2937e88ab87941a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spec Traceability" sheetId="4" r:id="R262d966e406948c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -125,21 +125,21 @@
   <x:dxfs count="4">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -844,9 +844,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O9" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P9" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P9" s="15" t="str">
+        <x:v>Owner manual production retest PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="15" t="str">
@@ -940,9 +942,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O11" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P11" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P11" s="15" t="str">
+        <x:v>Owner manual production retest PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="15" t="str">
@@ -1132,9 +1136,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O15" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P15" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P15" s="15" t="str">
+        <x:v>Owner manual production retest PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="15" t="str">
@@ -1276,9 +1282,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O18" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P18" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P18" s="15" t="str">
+        <x:v>Owner manual production retest PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="15" t="str">
@@ -1372,9 +1380,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O20" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P20" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P20" s="15" t="str">
+        <x:v>Owner manual production retest PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="15" t="str">
@@ -1612,9 +1622,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O25" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P25" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P25" s="15" t="str">
+        <x:v>Automated local account-separation regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="15" t="str">
@@ -1660,9 +1672,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O26" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P26" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P26" s="15" t="str">
+        <x:v>Automated local account-separation regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="15" t="str">
@@ -3772,9 +3786,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O70" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P70" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P70" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="15" t="str">
@@ -3820,9 +3836,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O71" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P71" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P71" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="15" t="str">
@@ -3868,9 +3886,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O72" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P72" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P72" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="15" t="str">
@@ -3916,9 +3936,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O73" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P73" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P73" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="15" t="str">
@@ -3964,9 +3986,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O74" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P74" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P74" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="15" t="str">
@@ -4012,9 +4036,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O75" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P75" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P75" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="15" t="str">
@@ -4060,9 +4086,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O76" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P76" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P76" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="15" t="str">
@@ -4108,9 +4136,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O77" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P77" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P77" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="15" t="str">
@@ -4156,9 +4186,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O78" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P78" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P78" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="15" t="str">
@@ -4204,9 +4236,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O79" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P79" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P79" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="15" t="str">
@@ -4252,9 +4286,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O80" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P80" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P80" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="15" t="str">
@@ -4300,9 +4336,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O81" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P81" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P81" s="15" t="str">
+        <x:v>Automated local SQL/RLS regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="15" t="str">
@@ -6604,9 +6642,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O129" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P129" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P129" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="15" t="str">
@@ -6652,9 +6692,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O130" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P130" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P130" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="15" t="str">
@@ -6700,9 +6742,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O131" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P131" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P131" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="15" t="str">
@@ -6748,9 +6792,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O132" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P132" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P132" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="15" t="str">
@@ -6796,9 +6842,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O133" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P133" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P133" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="15" t="str">
@@ -6844,9 +6892,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O134" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P134" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P134" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="15" t="str">
@@ -6892,9 +6942,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O135" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P135" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P135" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="15" t="str">
@@ -6940,9 +6992,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O136" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P136" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P136" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="15" t="str">
@@ -6988,9 +7042,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O137" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P137" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P137" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="15" t="str">
@@ -7036,9 +7092,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O138" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P138" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P138" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="15" t="str">
@@ -7084,9 +7142,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O139" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P139" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P139" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="15" t="str">
@@ -7132,9 +7192,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O140" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P140" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P140" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="15" t="str">
@@ -7180,9 +7242,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O141" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P141" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P141" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="15" t="str">
@@ -7228,9 +7292,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O142" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P142" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P142" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="15" t="str">
@@ -7276,9 +7342,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O143" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P143" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P143" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="15" t="str">
@@ -7324,9 +7392,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O144" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P144" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P144" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="15" t="str">
@@ -7372,9 +7442,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O145" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P145" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P145" s="15" t="str">
+        <x:v>Automated local SQL/API integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="15" t="str">
@@ -7420,9 +7492,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O146" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P146" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P146" s="15" t="str">
+        <x:v>Automated local SQL/integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="15" t="str">
@@ -7468,9 +7542,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O147" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P147" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P147" s="15" t="str">
+        <x:v>Automated local SQL/integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="15" t="str">
@@ -7516,9 +7592,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O148" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P148" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P148" s="15" t="str">
+        <x:v>Automated local SQL/integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="15" t="str">
@@ -7564,9 +7642,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O149" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P149" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P149" s="15" t="str">
+        <x:v>Automated local SQL/integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="15" t="str">
@@ -7612,9 +7692,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O150" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P150" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P150" s="15" t="str">
+        <x:v>Automated local SQL/integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="15" t="str">
@@ -7660,9 +7742,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O151" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P151" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P151" s="15" t="str">
+        <x:v>Automated local SQL/integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="15" t="str">
@@ -7708,9 +7792,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O152" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P152" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P152" s="15" t="str">
+        <x:v>Automated local SQL/integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="15" t="str">
@@ -7756,9 +7842,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O153" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P153" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P153" s="15" t="str">
+        <x:v>Automated local SQL/integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="15" t="str">
@@ -7804,9 +7892,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O154" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P154" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P154" s="15" t="str">
+        <x:v>Automated local SQL/integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="15" t="str">
@@ -7852,9 +7942,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O155" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P155" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P155" s="15" t="str">
+        <x:v>Automated local SQL/integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="15" t="str">
@@ -7900,9 +7992,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O156" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P156" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P156" s="15" t="str">
+        <x:v>Automated local SQL/integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="15" t="str">
@@ -7948,9 +8042,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O157" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P157" s="15" t="str"/>
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="P157" s="15" t="str">
+        <x:v>Owner manual browser QA required after deployment — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="15" t="str">
@@ -7996,9 +8092,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O158" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P158" s="15" t="str"/>
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="P158" s="15" t="str">
+        <x:v>Owner manual browser QA required after deployment — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="15" t="str">
@@ -8044,9 +8142,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O159" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P159" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P159" s="15" t="str">
+        <x:v>Automated local SQL/concurrency integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="15" t="str">
@@ -8092,9 +8192,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O160" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P160" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P160" s="15" t="str">
+        <x:v>Automated local SQL/concurrency integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="15" t="str">
@@ -8140,9 +8242,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O161" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P161" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P161" s="15" t="str">
+        <x:v>Automated local SQL/concurrency integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="15" t="str">
@@ -8188,9 +8292,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O162" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P162" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P162" s="15" t="str">
+        <x:v>Automated local SQL/concurrency integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="15" t="str">
@@ -8236,9 +8342,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O163" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P163" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P163" s="15" t="str">
+        <x:v>Automated local SQL/concurrency integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="15" t="str">
@@ -8284,9 +8392,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O164" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P164" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P164" s="15" t="str">
+        <x:v>Automated local SQL/concurrency integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="15" t="str">
@@ -8332,9 +8442,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O165" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P165" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P165" s="15" t="str">
+        <x:v>Automated local SQL/concurrency integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="15" t="str">
@@ -8380,9 +8492,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O166" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P166" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P166" s="15" t="str">
+        <x:v>Automated local SQL/concurrency integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="15" t="str">
@@ -8428,9 +8542,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O167" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P167" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P167" s="15" t="str">
+        <x:v>Automated local SQL/concurrency integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="15" t="str">
@@ -8476,9 +8592,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O168" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P168" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P168" s="15" t="str">
+        <x:v>Automated local SQL/concurrency integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="15" t="str">
@@ -8524,9 +8642,11 @@
         <x:v>BUILD</x:v>
       </x:c>
       <x:c r="O169" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P169" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P169" s="15" t="str">
+        <x:v>Automated local SQL/concurrency integration PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="15" t="str">
@@ -14524,9 +14644,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O294" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P294" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P294" s="15" t="str">
+        <x:v>Owner production/manual regression PASS; Sprint 2 checks preserved — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="295">
       <x:c r="A295" s="15" t="str">
@@ -14908,9 +15030,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O302" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P302" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P302" s="15" t="str">
+        <x:v>Automated local SQL/RLS compatibility PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="303">
       <x:c r="A303" s="15" t="str">
@@ -15100,9 +15224,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O306" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P306" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P306" s="15" t="str">
+        <x:v>Automated local SQL/RLS compatibility PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="307">
       <x:c r="A307" s="15" t="str">
@@ -15196,9 +15322,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O308" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P308" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P308" s="15" t="str">
+        <x:v>Automated local SQL/RLS compatibility PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="309">
       <x:c r="A309" s="15" t="str">
@@ -15244,9 +15372,11 @@
         <x:v>MODIFY</x:v>
       </x:c>
       <x:c r="O309" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P309" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P309" s="15" t="str">
+        <x:v>Owner production/manual regression PASS; Sprint 2 checks preserved — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="310">
       <x:c r="A310" s="15" t="str">
@@ -16156,9 +16286,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O328" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P328" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P328" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="329">
       <x:c r="A329" s="15" t="str">
@@ -16204,9 +16336,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O329" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P329" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P329" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="330">
       <x:c r="A330" s="15" t="str">
@@ -16252,9 +16386,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O330" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P330" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P330" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="331">
       <x:c r="A331" s="15" t="str">
@@ -16300,9 +16436,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O331" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P331" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P331" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="332">
       <x:c r="A332" s="15" t="str">
@@ -16348,9 +16486,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O332" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P332" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P332" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="333">
       <x:c r="A333" s="15" t="str">
@@ -16396,9 +16536,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O333" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P333" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P333" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="334">
       <x:c r="A334" s="15" t="str">
@@ -16444,9 +16586,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O334" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P334" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P334" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="335">
       <x:c r="A335" s="15" t="str">
@@ -16492,9 +16636,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O335" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P335" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P335" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="336">
       <x:c r="A336" s="15" t="str">
@@ -16540,9 +16686,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O336" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P336" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P336" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="337">
       <x:c r="A337" s="15" t="str">
@@ -16588,9 +16736,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O337" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P337" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P337" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="338">
       <x:c r="A338" s="15" t="str">
@@ -16636,9 +16786,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O338" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P338" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P338" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="339">
       <x:c r="A339" s="15" t="str">
@@ -16684,9 +16836,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O339" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P339" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P339" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="340">
       <x:c r="A340" s="15" t="str">
@@ -16732,9 +16886,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O340" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P340" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P340" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="341">
       <x:c r="A341" s="15" t="str">
@@ -16780,9 +16936,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O341" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P341" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P341" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="342">
       <x:c r="A342" s="15" t="str">
@@ -16828,9 +16986,11 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="O342" s="15" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="P342" s="15" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="P342" s="15" t="str">
+        <x:v>Automated local regression PASS — 2026-09-10</x:v>
+      </x:c>
     </x:row>
     <x:row r="343">
       <x:c r="A343" s="15" t="str">
@@ -17249,7 +17409,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90ae8ff4ffc24c27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda49dbaba0a24b9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17419,7 +17579,7 @@
       </x:c>
       <x:c r="B10" s="12" t="n">
         <x:f>COUNTIF('Acceptance Matrix'!O2:O350,"Pass")</x:f>
-        <x:v>0</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
         <x:v>Stores</x:v>
@@ -17786,7 +17946,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb2fe027e2ac476f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fb3748f2e1146e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18126,7 +18286,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64ccdf66fc0d4447"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reaf06f0db1c748e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>